<commit_message>
Close five documentation gaps in tranche A
Found uncommitted in the working tree at the start of this session, not produced
by it. Committed as its own change so its provenance stays separate.

DOGE burn, DOGE capture, LTC burn, HBAR burn and OP burn resolve to No against
dated primary sources, archived under data/raw/classification_sources/2026-09-14.
OP capture stays pending: execution reports confirm three completed buybacks but
do not establish continued operation at the classification date.

Evidence-backed cells 119 to 124, pending 11 to 6, provisional unchanged at 120.
No independent review was added.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNFXB4FbiDjTqSf2G6dTLQ
</commit_message>
<xml_diff>
--- a/data/reference/digital_asset_research_universe.xlsx
+++ b/data/reference/digital_asset_research_universe.xlsx
@@ -656,7 +656,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>109 — dated primary source, NOT independently reviewed</t>
+          <t>114 — dated primary source, NOT independently reviewed</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>11 — held for adjudication</t>
+          <t>6 — held for adjudication</t>
         </is>
       </c>
     </row>
@@ -1316,10 +1316,10 @@
       </c>
       <c r="K12" s="7" t="n"/>
       <c r="L12" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M12" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N12" s="7" t="n">
         <v>5</v>
@@ -1730,10 +1730,10 @@
       </c>
       <c r="K19" s="7" t="n"/>
       <c r="L19" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M19" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N19" s="7" t="n">
         <v>5</v>
@@ -1790,11 +1790,9 @@
       </c>
       <c r="K20" s="7" t="n"/>
       <c r="L20" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="M20" s="7" t="n">
-        <v>1</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="M20" s="7" t="n"/>
       <c r="N20" s="7" t="n">
         <v>5</v>
       </c>
@@ -2228,10 +2226,10 @@
       <c r="J28" s="7" t="n"/>
       <c r="K28" s="7" t="n"/>
       <c r="L28" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M28" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N28" s="7" t="n">
         <v>5</v>
@@ -3654,7 +3652,9 @@
       <c r="F12" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="21" t="n"/>
+      <c r="G12" s="16" t="n">
+        <v>0</v>
+      </c>
       <c r="H12" s="16" t="n">
         <v>0</v>
       </c>
@@ -3664,7 +3664,9 @@
       <c r="J12" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="21" t="n"/>
+      <c r="K12" s="16" t="n">
+        <v>0</v>
+      </c>
       <c r="L12" s="20" t="n">
         <v>0</v>
       </c>
@@ -3676,7 +3678,7 @@
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>3 pending</t>
+          <t>1 pending</t>
         </is>
       </c>
     </row>
@@ -3999,7 +4001,9 @@
       <c r="F19" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="21" t="n"/>
+      <c r="G19" s="16" t="n">
+        <v>0</v>
+      </c>
       <c r="H19" s="15" t="n">
         <v>1</v>
       </c>
@@ -4023,7 +4027,7 @@
       </c>
       <c r="O19" s="7" t="inlineStr">
         <is>
-          <t>2 pending</t>
+          <t>1 pending</t>
         </is>
       </c>
     </row>
@@ -4048,7 +4052,9 @@
       <c r="F20" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="21" t="n"/>
+      <c r="G20" s="16" t="n">
+        <v>0</v>
+      </c>
       <c r="H20" s="15" t="n">
         <v>1</v>
       </c>
@@ -4072,7 +4078,7 @@
       </c>
       <c r="O20" s="7" t="inlineStr">
         <is>
-          <t>1 pending</t>
+          <t>mixed</t>
         </is>
       </c>
     </row>
@@ -4466,7 +4472,9 @@
       <c r="F28" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="G28" s="21" t="n"/>
+      <c r="G28" s="16" t="n">
+        <v>0</v>
+      </c>
       <c r="H28" s="16" t="n">
         <v>0</v>
       </c>
@@ -4488,7 +4496,7 @@
       </c>
       <c r="O28" s="7" t="inlineStr">
         <is>
-          <t>2 pending</t>
+          <t>1 pending</t>
         </is>
       </c>
     </row>
@@ -6865,10 +6873,12 @@
           <t>VA_BURN</t>
         </is>
       </c>
-      <c r="C64" s="30" t="n"/>
+      <c r="C64" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="D64" s="30" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E64" s="30" t="inlineStr">
@@ -6878,7 +6888,7 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>https://dogecoin.com/dogepedia/faq/putting-a-cap-on-dogecoin/</t>
+          <t>https://dogecoin.com/dogepedia/articles/what-is-a-miner/</t>
         </is>
       </c>
     </row>
@@ -6921,10 +6931,12 @@
           <t>VA_PROTOCOL</t>
         </is>
       </c>
-      <c r="C66" s="30" t="n"/>
+      <c r="C66" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="D66" s="30" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E66" s="30" t="inlineStr">
@@ -6934,7 +6946,7 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>https://dogecoin.com/dogepedia/faq/putting-a-cap-on-dogecoin/</t>
+          <t>https://dogecoin.com/dogepedia/articles/what-is-a-miner/</t>
         </is>
       </c>
     </row>
@@ -7309,10 +7321,12 @@
           <t>VA_BURN</t>
         </is>
       </c>
-      <c r="C79" s="30" t="n"/>
+      <c r="C79" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="D79" s="30" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="E79" s="30" t="inlineStr">
@@ -7322,7 +7336,7 @@
       </c>
       <c r="F79" s="30" t="inlineStr">
         <is>
-          <t>https://docs.hedera.com/hedera/networks/mainnet/fees</t>
+          <t>https://hedera.com/terms/</t>
         </is>
       </c>
     </row>
@@ -7605,10 +7619,12 @@
           <t>VA_BURN</t>
         </is>
       </c>
-      <c r="C89" s="30" t="n"/>
+      <c r="C89" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="D89" s="30" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E89" s="30" t="inlineStr">
@@ -7751,10 +7767,12 @@
           <t>VA_BURN</t>
         </is>
       </c>
-      <c r="C94" s="30" t="n"/>
+      <c r="C94" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="D94" s="30" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="E94" s="30" t="inlineStr">
@@ -7764,7 +7782,7 @@
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>https://specs.optimism.io/experimental/gov-token.html</t>
+          <t>https://optimism.io/blog/op-token-buybacks</t>
         </is>
       </c>
     </row>
@@ -7812,7 +7830,7 @@
       <c r="C96" s="30" t="n"/>
       <c r="D96" s="30" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E96" s="30" t="inlineStr">

</xml_diff>